<commit_message>
feat: todos los cambios recientes en dashboard, favicon, badge dinámico, y despliegue GitHub Pages
</commit_message>
<xml_diff>
--- a/Presentación Semanal UAT.xlsx
+++ b/Presentación Semanal UAT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\QA\WrampUp - copia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76645C27-E99C-452D-A523-5E9B8498EDD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE1C8A8C-8FEF-4826-ABED-0E7D22787C70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{27A98AC9-9505-493B-985E-2D79FFCBCA40}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="50">
   <si>
     <t>Aplicación</t>
   </si>
@@ -158,9 +158,6 @@
     <t>Remesas</t>
   </si>
   <si>
-    <t>Compra y Venta de Dolares</t>
-  </si>
-  <si>
     <t>Depósitos/Retiros/Transferencias</t>
   </si>
   <si>
@@ -174,6 +171,27 @@
   </si>
   <si>
     <t>TOTAL ABIERTOS</t>
+  </si>
+  <si>
+    <t>CONFIGURACIÓN</t>
+  </si>
+  <si>
+    <t>Mantenimiento Datos Cliente</t>
+  </si>
+  <si>
+    <t>Gestión de DPF</t>
+  </si>
+  <si>
+    <t>Gestión de Cuentas CTS</t>
+  </si>
+  <si>
+    <t>Compra y Venta de Dólares</t>
+  </si>
+  <si>
+    <t>Gestión de Préstamos</t>
+  </si>
+  <si>
+    <t>Simulación de Préstamos</t>
   </si>
 </sst>
 </file>
@@ -505,6 +523,50 @@
                 </c:ext>
               </c:extLst>
             </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-4.2868741542625169E-2"/>
+                  <c:y val="5.2667369928041288E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000001-81F2-4ACE-BA43-26898F74B067}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="3"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-4.0162381596752367E-2"/>
+                  <c:y val="6.2236747918471828E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000000-81F2-4ACE-BA43-26898F74B067}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -575,6 +637,9 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>144</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>129</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1047,6 +1112,9 @@
                 <c:pt idx="2">
                   <c:v>933</c:v>
                 </c:pt>
+                <c:pt idx="3">
+                  <c:v>904</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -3582,11 +3650,16 @@
         <f t="shared" si="0"/>
         <v>127</v>
       </c>
-      <c r="D5" s="6"/>
+      <c r="D5" s="6">
+        <f>D4-F5</f>
+        <v>129</v>
+      </c>
       <c r="E5" s="6">
-        <v>25</v>
-      </c>
-      <c r="F5" s="6"/>
+        <v>20</v>
+      </c>
+      <c r="F5" s="6">
+        <v>15</v>
+      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
@@ -3652,7 +3725,7 @@
       </c>
       <c r="D9" s="6"/>
       <c r="E9" s="6">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F9" s="6"/>
     </row>
@@ -3668,7 +3741,9 @@
         <v>2</v>
       </c>
       <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
+      <c r="E10" s="6">
+        <v>32</v>
+      </c>
       <c r="F10" s="6"/>
     </row>
   </sheetData>
@@ -3785,11 +3860,16 @@
         <f t="shared" si="0"/>
         <v>656</v>
       </c>
-      <c r="D5" s="6"/>
+      <c r="D5" s="6">
+        <f>D4-F5</f>
+        <v>904</v>
+      </c>
       <c r="E5" s="6">
         <v>131</v>
       </c>
-      <c r="F5" s="6"/>
+      <c r="F5" s="6">
+        <v>29</v>
+      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
@@ -3882,10 +3962,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A735EDFD-2DED-4B82-BC46-A3A7E7C548CD}">
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="28.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.1796875" bestFit="1" customWidth="1"/>
     <col min="3" max="10" width="10.90625" style="1"/>
   </cols>
   <sheetData>
@@ -3934,19 +4014,25 @@
       <c r="D2" s="1">
         <v>91</v>
       </c>
+      <c r="E2" s="1">
+        <v>87</v>
+      </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="C3" s="1">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="D3" s="1">
-        <v>37</v>
+        <v>0</v>
+      </c>
+      <c r="E3" s="1">
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
@@ -3954,13 +4040,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C4" s="1">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D4" s="1">
-        <v>16</v>
+        <v>37</v>
+      </c>
+      <c r="E4" s="1">
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
@@ -3968,13 +4057,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C5" s="1">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D5" s="1">
         <v>16</v>
+      </c>
+      <c r="E5" s="1">
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
@@ -3982,53 +4074,33 @@
         <v>1</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C6" s="1">
+        <v>8</v>
+      </c>
+      <c r="D6" s="1">
         <v>16</v>
       </c>
-      <c r="D6" s="1">
-        <v>30</v>
+      <c r="E6" s="1">
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" s="2">
-        <f>SUM(C2:C6)</f>
-        <v>119</v>
-      </c>
-      <c r="D7" s="2">
-        <f t="shared" ref="D7:J7" si="0">SUM(D2:D6)</f>
-        <v>190</v>
-      </c>
-      <c r="E7" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F7" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G7" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H7" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I7" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J7" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
+      <c r="B7" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="1">
+        <v>16</v>
+      </c>
+      <c r="D7" s="1">
+        <v>30</v>
+      </c>
+      <c r="E7" s="1">
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
@@ -4036,85 +4108,111 @@
         <v>1</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="C8" s="2">
-        <f>SUM(C2:C6)-C6</f>
+        <f>SUM(C2:C7)</f>
+        <v>119</v>
+      </c>
+      <c r="D8" s="2">
+        <f t="shared" ref="D8:J8" si="0">SUM(D2:D7)</f>
+        <v>190</v>
+      </c>
+      <c r="E8" s="2">
+        <f t="shared" si="0"/>
+        <v>258</v>
+      </c>
+      <c r="F8" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G8" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H8" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I8" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J8" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="2">
+        <f>SUM(C2:C7)-C7</f>
         <v>103</v>
       </c>
-      <c r="D8" s="2">
-        <f t="shared" ref="D8:J8" si="1">SUM(D2:D6)-D6</f>
+      <c r="D9" s="2">
+        <f t="shared" ref="D9:J9" si="1">SUM(D2:D7)-D7</f>
         <v>160</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E9" s="2">
+        <f>SUM(E2:E7)-E7</f>
+        <v>220</v>
+      </c>
+      <c r="F9" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="F8" s="2">
+      <c r="G9" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G8" s="2">
+      <c r="H9" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H8" s="2">
+      <c r="I9" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I8" s="2">
+      <c r="J9" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J8" s="2">
-        <f t="shared" si="1"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" s="9" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A10" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B10" s="9" t="s">
+      <c r="B11" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F11" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H11" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="I11" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="J11" s="2" t="s">
         <v>33</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>1</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="C11" s="1">
-        <v>23</v>
-      </c>
-      <c r="D11" s="1">
-        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
@@ -4122,13 +4220,16 @@
         <v>1</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C12" s="1">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="D12" s="1">
-        <v>5</v>
+        <v>23</v>
+      </c>
+      <c r="E12" s="1">
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
@@ -4136,13 +4237,16 @@
         <v>1</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C13" s="1">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="D13" s="1">
-        <v>14</v>
+        <v>5</v>
+      </c>
+      <c r="E13" s="1">
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
@@ -4150,13 +4254,16 @@
         <v>1</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C14" s="1">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D14" s="1">
-        <v>7</v>
+        <v>14</v>
+      </c>
+      <c r="E14" s="1">
+        <v>16</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
@@ -4164,13 +4271,16 @@
         <v>1</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="C15" s="1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D15" s="1">
-        <v>4</v>
+        <v>7</v>
+      </c>
+      <c r="E15" s="1">
+        <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
@@ -4178,13 +4288,16 @@
         <v>1</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C16" s="1">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D16" s="1">
-        <v>7</v>
+        <v>4</v>
+      </c>
+      <c r="E16" s="1">
+        <v>9</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
@@ -4192,13 +4305,16 @@
         <v>1</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C17" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D17" s="1">
-        <v>4</v>
+        <v>7</v>
+      </c>
+      <c r="E17" s="1">
+        <v>18</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
@@ -4206,13 +4322,16 @@
         <v>1</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C18" s="1">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="D18" s="1">
-        <v>96</v>
+        <v>4</v>
+      </c>
+      <c r="E18" s="1">
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
@@ -4220,92 +4339,197 @@
         <v>1</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="C19" s="1">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="D19" s="1">
-        <v>30</v>
+        <v>0</v>
+      </c>
+      <c r="E19" s="1">
+        <v>7</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>1</v>
       </c>
-      <c r="B20" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="C20" s="2">
-        <f>SUM(C11:C19)</f>
-        <v>119</v>
-      </c>
-      <c r="D20" s="2">
-        <f>SUM(D11:D19)</f>
-        <v>190</v>
-      </c>
-      <c r="E20" s="2">
-        <f t="shared" ref="E20" si="2">SUM(E14:E18)</f>
+      <c r="B20" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="1">
         <v>0</v>
       </c>
-      <c r="F20" s="2">
-        <f t="shared" ref="F20" si="3">SUM(F14:F18)</f>
+      <c r="D20" s="1">
         <v>0</v>
       </c>
-      <c r="G20" s="2">
-        <f t="shared" ref="G20" si="4">SUM(G14:G18)</f>
-        <v>0</v>
-      </c>
-      <c r="H20" s="2">
-        <f t="shared" ref="H20" si="5">SUM(H14:H18)</f>
-        <v>0</v>
-      </c>
-      <c r="I20" s="2">
-        <f t="shared" ref="I20" si="6">SUM(I14:I18)</f>
-        <v>0</v>
-      </c>
-      <c r="J20" s="2">
-        <f t="shared" ref="J20" si="7">SUM(J14:J18)</f>
-        <v>0</v>
+      <c r="E20" s="1">
+        <v>23</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>1</v>
       </c>
-      <c r="B21" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="C21" s="2">
-        <f>SUM(C11:C19)-C19</f>
+      <c r="B21" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C21" s="1">
+        <v>0</v>
+      </c>
+      <c r="D21" s="1">
+        <v>0</v>
+      </c>
+      <c r="E21" s="1">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>1</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C22" s="1">
+        <v>0</v>
+      </c>
+      <c r="D22" s="1">
+        <v>0</v>
+      </c>
+      <c r="E22" s="1">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>1</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C23" s="1">
+        <v>0</v>
+      </c>
+      <c r="D23" s="1">
+        <v>0</v>
+      </c>
+      <c r="E23" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>1</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C24" s="1">
+        <v>40</v>
+      </c>
+      <c r="D24" s="1">
+        <v>96</v>
+      </c>
+      <c r="E24" s="1">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>1</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C25" s="1">
+        <v>16</v>
+      </c>
+      <c r="D25" s="1">
+        <v>30</v>
+      </c>
+      <c r="E25" s="1">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>1</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C26" s="2">
+        <f>SUM(C12:C25)</f>
+        <v>119</v>
+      </c>
+      <c r="D26" s="2">
+        <f>SUM(D12:D25)</f>
+        <v>190</v>
+      </c>
+      <c r="E26" s="2">
+        <f>SUM(E12:E25)</f>
+        <v>258</v>
+      </c>
+      <c r="F26" s="2">
+        <f t="shared" ref="F26" si="2">SUM(F15:F24)</f>
+        <v>0</v>
+      </c>
+      <c r="G26" s="2">
+        <f t="shared" ref="G26" si="3">SUM(G15:G24)</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="2">
+        <f t="shared" ref="H26" si="4">SUM(H15:H24)</f>
+        <v>0</v>
+      </c>
+      <c r="I26" s="2">
+        <f t="shared" ref="I26" si="5">SUM(I15:I24)</f>
+        <v>0</v>
+      </c>
+      <c r="J26" s="2">
+        <f t="shared" ref="J26" si="6">SUM(J15:J24)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>1</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C27" s="2">
+        <f>SUM(C12:C25)-C25</f>
         <v>103</v>
       </c>
-      <c r="D21" s="2">
-        <f>SUM(D11:D19)-D19</f>
+      <c r="D27" s="2">
+        <f>SUM(D12:D25)-D25</f>
         <v>160</v>
       </c>
-      <c r="E21" s="2">
-        <f t="shared" ref="E21:J21" si="8">SUM(E14:E18)-E18</f>
+      <c r="E27" s="2">
+        <f>SUM(E12:E25)-E25</f>
+        <v>220</v>
+      </c>
+      <c r="F27" s="2">
+        <f t="shared" ref="E27:J27" si="7">SUM(F15:F24)-F24</f>
         <v>0</v>
       </c>
-      <c r="F21" s="2">
-        <f t="shared" si="8"/>
+      <c r="G27" s="2">
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="G21" s="2">
-        <f t="shared" si="8"/>
+      <c r="H27" s="2">
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="H21" s="2">
-        <f t="shared" si="8"/>
+      <c r="I27" s="2">
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="I21" s="2">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="J21" s="2">
-        <f t="shared" si="8"/>
+      <c r="J27" s="2">
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: pestaña Observaciones Críticas con tabla completa, columnas ajustadas y datos estáticos
</commit_message>
<xml_diff>
--- a/Presentación Semanal UAT.xlsx
+++ b/Presentación Semanal UAT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\QA\WrampUp - copia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE1C8A8C-8FEF-4826-ABED-0E7D22787C70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E571F51-14C2-4EAF-A1A6-1D6523B036B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{27A98AC9-9505-493B-985E-2D79FFCBCA40}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{27A98AC9-9505-493B-985E-2D79FFCBCA40}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="49">
   <si>
     <t>Aplicación</t>
   </si>
@@ -71,127 +71,124 @@
     <t>ODS SPACE - IVR</t>
   </si>
   <si>
-    <t>ODS SPACE - Reclamos</t>
-  </si>
-  <si>
-    <t>TBD</t>
+    <t>2 Semanas</t>
+  </si>
+  <si>
+    <t>Semana</t>
+  </si>
+  <si>
+    <t>Proyectado</t>
+  </si>
+  <si>
+    <t>Real</t>
+  </si>
+  <si>
+    <t>Diario Real</t>
+  </si>
+  <si>
+    <t>Semanal Proyectado</t>
+  </si>
+  <si>
+    <t>Semanal Real</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>WORK IN PROGRESS</t>
+  </si>
+  <si>
+    <t>RESUELTOS</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t>Semana 1</t>
+  </si>
+  <si>
+    <t>Semana 2</t>
+  </si>
+  <si>
+    <t>Semana 3</t>
+  </si>
+  <si>
+    <t>Semana 4</t>
+  </si>
+  <si>
+    <t>Semana 5</t>
+  </si>
+  <si>
+    <t>Semana 6</t>
+  </si>
+  <si>
+    <t>Semana 7</t>
+  </si>
+  <si>
+    <t>Semana 8</t>
+  </si>
+  <si>
+    <t>Grupos Funcionales</t>
+  </si>
+  <si>
+    <t>Arqueo y Cierre de Caja</t>
+  </si>
+  <si>
+    <t>Boveda</t>
+  </si>
+  <si>
+    <t>Remesas</t>
+  </si>
+  <si>
+    <t>Depósitos/Retiros/Transferencias</t>
+  </si>
+  <si>
+    <t>Gestión de Cuentas de Ahorro</t>
+  </si>
+  <si>
+    <t>Perfilamiento</t>
+  </si>
+  <si>
+    <t>TOTAL ABIERTOS</t>
+  </si>
+  <si>
+    <t>Mantenimiento Datos Cliente</t>
+  </si>
+  <si>
+    <t>Gestión de DPF</t>
+  </si>
+  <si>
+    <t>Gestión de Cuentas CTS</t>
+  </si>
+  <si>
+    <t>Compra y Venta de Dólares</t>
+  </si>
+  <si>
+    <t>Gestión de Préstamos</t>
+  </si>
+  <si>
+    <t>Simulación de Préstamos</t>
+  </si>
+  <si>
+    <t>ISSUE</t>
+  </si>
+  <si>
+    <t>DEFECTO FUNCIONAL</t>
+  </si>
+  <si>
+    <t>GAP DE PAQUETE</t>
+  </si>
+  <si>
+    <t>NO APLICA</t>
+  </si>
+  <si>
+    <t>DEFECTO PARAMETRÍA</t>
   </si>
   <si>
     <t>8 Semanas</t>
   </si>
   <si>
-    <t>2 Semanas</t>
-  </si>
-  <si>
-    <t>Semana</t>
-  </si>
-  <si>
-    <t>Proyectado</t>
-  </si>
-  <si>
-    <t>Real</t>
-  </si>
-  <si>
-    <t>Diario Real</t>
-  </si>
-  <si>
-    <t>Semanal Proyectado</t>
-  </si>
-  <si>
-    <t>Semanal Real</t>
-  </si>
-  <si>
-    <t>Estado</t>
-  </si>
-  <si>
-    <t>WORK IN PROGRESS</t>
-  </si>
-  <si>
-    <t>CAMBIO DE ALCANCE</t>
-  </si>
-  <si>
-    <t>GAP DE REQUERIMIENTO</t>
-  </si>
-  <si>
-    <t>DEFECTOS</t>
-  </si>
-  <si>
-    <t>RESUELTOS</t>
-  </si>
-  <si>
-    <t>TOTAL</t>
-  </si>
-  <si>
-    <t>Semana 1</t>
-  </si>
-  <si>
-    <t>Semana 2</t>
-  </si>
-  <si>
-    <t>Semana 3</t>
-  </si>
-  <si>
-    <t>Semana 4</t>
-  </si>
-  <si>
-    <t>Semana 5</t>
-  </si>
-  <si>
-    <t>Semana 6</t>
-  </si>
-  <si>
-    <t>Semana 7</t>
-  </si>
-  <si>
-    <t>Semana 8</t>
-  </si>
-  <si>
-    <t>Grupos Funcionales</t>
-  </si>
-  <si>
-    <t>Arqueo y Cierre de Caja</t>
-  </si>
-  <si>
-    <t>Boveda</t>
-  </si>
-  <si>
-    <t>Remesas</t>
-  </si>
-  <si>
-    <t>Depósitos/Retiros/Transferencias</t>
-  </si>
-  <si>
-    <t>Gestión de Cuentas de Ahorro</t>
-  </si>
-  <si>
-    <t>Perfilamiento</t>
-  </si>
-  <si>
-    <t>Otros</t>
-  </si>
-  <si>
-    <t>TOTAL ABIERTOS</t>
-  </si>
-  <si>
-    <t>CONFIGURACIÓN</t>
-  </si>
-  <si>
-    <t>Mantenimiento Datos Cliente</t>
-  </si>
-  <si>
-    <t>Gestión de DPF</t>
-  </si>
-  <si>
-    <t>Gestión de Cuentas CTS</t>
-  </si>
-  <si>
-    <t>Compra y Venta de Dólares</t>
-  </si>
-  <si>
-    <t>Gestión de Préstamos</t>
-  </si>
-  <si>
-    <t>Simulación de Préstamos</t>
+    <t>ODS SPACE - Reclamos y Dalis</t>
   </si>
 </sst>
 </file>
@@ -229,7 +226,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -239,6 +236,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC00000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -270,7 +273,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -293,6 +296,10 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -426,28 +433,28 @@
                   <c:v>202</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>177</c:v>
+                  <c:v>179</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>152</c:v>
+                  <c:v>156</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>127</c:v>
+                  <c:v>133</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>102</c:v>
+                  <c:v>110</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>77</c:v>
+                  <c:v>87</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>52</c:v>
+                  <c:v>64</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>27</c:v>
+                  <c:v>41</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2</c:v>
+                  <c:v>18</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -640,6 +647,9 @@
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>129</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>116</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -966,28 +976,28 @@
                   <c:v>1049</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>918</c:v>
+                  <c:v>933</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>787</c:v>
+                  <c:v>817</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>656</c:v>
+                  <c:v>701</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>525</c:v>
+                  <c:v>585</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>394</c:v>
+                  <c:v>469</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>263</c:v>
+                  <c:v>353</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>132</c:v>
+                  <c:v>237</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1</c:v>
+                  <c:v>121</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1114,6 +1124,9 @@
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>904</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>874</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3424,7 +3437,7 @@
   <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.36328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.36328125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.90625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.81640625" style="1" bestFit="1" customWidth="1"/>
@@ -3470,7 +3483,7 @@
         <v>1049</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>11</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
@@ -3491,7 +3504,7 @@
         <v>74</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
@@ -3502,38 +3515,38 @@
         <v>82</v>
       </c>
       <c r="C4" s="6">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D4" s="7">
         <f t="shared" ref="D4:D5" si="0">(C4*100)/B4</f>
-        <v>9.7560975609756095</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>10</v>
+        <v>8.536585365853659</v>
+      </c>
+      <c r="E4" s="6">
+        <v>161</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="s">
-        <v>9</v>
+        <v>48</v>
       </c>
       <c r="B5" s="11">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="C5" s="6">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D5" s="7">
         <f t="shared" si="0"/>
-        <v>26.086956521739129</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>10</v>
+        <v>21.621621621621621</v>
+      </c>
+      <c r="E5" s="6">
+        <v>47</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -3544,7 +3557,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42DF1849-A1A9-4E05-97A1-E2B79B421503}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.36328125" bestFit="1" customWidth="1"/>
@@ -3557,41 +3570,41 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E1" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>18</v>
-      </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="5">
+      <c r="A2" s="12">
         <v>0</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="6">
+      <c r="B2" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="13">
         <v>202</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="13">
         <v>202</v>
       </c>
-      <c r="E2" s="6">
-        <v>25</v>
-      </c>
-      <c r="F2" s="6">
+      <c r="E2" s="13">
+        <v>23</v>
+      </c>
+      <c r="F2" s="13">
         <v>0</v>
       </c>
     </row>
@@ -3604,14 +3617,14 @@
       </c>
       <c r="C3" s="6">
         <f>C2-$E$2</f>
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="D3" s="6">
         <f>D2-F3</f>
         <v>164</v>
       </c>
       <c r="E3" s="6">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F3" s="6">
         <v>38</v>
@@ -3625,15 +3638,15 @@
         <v>1</v>
       </c>
       <c r="C4" s="6">
-        <f t="shared" ref="C4:C10" si="0">C3-$E$2</f>
-        <v>152</v>
+        <f>C3-$E$2</f>
+        <v>156</v>
       </c>
       <c r="D4" s="6">
         <f>D3-F4</f>
         <v>144</v>
       </c>
       <c r="E4" s="6">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F4" s="6">
         <v>20</v>
@@ -3647,8 +3660,8 @@
         <v>1</v>
       </c>
       <c r="C5" s="6">
-        <f t="shared" si="0"/>
-        <v>127</v>
+        <f t="shared" ref="C5:C11" si="0">C4-$E$2</f>
+        <v>133</v>
       </c>
       <c r="D5" s="6">
         <f>D4-F5</f>
@@ -3670,13 +3683,18 @@
       </c>
       <c r="C6" s="6">
         <f t="shared" si="0"/>
-        <v>102</v>
-      </c>
-      <c r="D6" s="6"/>
+        <v>110</v>
+      </c>
+      <c r="D6" s="6">
+        <f>D5-F6</f>
+        <v>116</v>
+      </c>
       <c r="E6" s="6">
-        <v>25</v>
-      </c>
-      <c r="F6" s="6"/>
+        <v>20</v>
+      </c>
+      <c r="F6" s="6">
+        <v>13</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
@@ -3687,11 +3705,11 @@
       </c>
       <c r="C7" s="6">
         <f t="shared" si="0"/>
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="D7" s="6"/>
       <c r="E7" s="6">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F7" s="6"/>
     </row>
@@ -3704,11 +3722,11 @@
       </c>
       <c r="C8" s="6">
         <f t="shared" si="0"/>
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="D8" s="6"/>
       <c r="E8" s="6">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F8" s="6"/>
     </row>
@@ -3721,11 +3739,11 @@
       </c>
       <c r="C9" s="6">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="D9" s="6"/>
       <c r="E9" s="6">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F9" s="6"/>
     </row>
@@ -3738,13 +3756,30 @@
       </c>
       <c r="C10" s="6">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="6">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="F10" s="6"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" s="5">
+        <v>9</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C11" s="6">
+        <f t="shared" si="0"/>
+        <v>-5</v>
+      </c>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6">
+        <v>24</v>
+      </c>
+      <c r="F11" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3754,7 +3789,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20BCB52B-56FF-4E38-A246-A8F336FD8B79}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.36328125" bestFit="1" customWidth="1"/>
@@ -3767,41 +3802,41 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>17</v>
-      </c>
       <c r="F1" s="4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="5">
+      <c r="A2" s="12">
         <v>0</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="6">
+      <c r="B2" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="13">
         <v>1049</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="13">
         <v>1049</v>
       </c>
-      <c r="E2" s="6">
-        <v>131</v>
-      </c>
-      <c r="F2" s="6">
+      <c r="E2" s="13">
+        <v>116</v>
+      </c>
+      <c r="F2" s="13">
         <v>0</v>
       </c>
     </row>
@@ -3814,14 +3849,14 @@
       </c>
       <c r="C3" s="6">
         <f>C2-$E$2</f>
-        <v>918</v>
+        <v>933</v>
       </c>
       <c r="D3" s="6">
         <f>D2-F3</f>
         <v>983</v>
       </c>
       <c r="E3" s="6">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="F3" s="6">
         <v>66</v>
@@ -3835,15 +3870,15 @@
         <v>1</v>
       </c>
       <c r="C4" s="6">
-        <f t="shared" ref="C4:C10" si="0">C3-$E$2</f>
-        <v>787</v>
+        <f t="shared" ref="C4:C11" si="0">C3-$E$2</f>
+        <v>817</v>
       </c>
       <c r="D4" s="6">
         <f>D3-F4</f>
         <v>933</v>
       </c>
       <c r="E4" s="6">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="F4" s="6">
         <v>50</v>
@@ -3858,14 +3893,14 @@
       </c>
       <c r="C5" s="6">
         <f t="shared" si="0"/>
-        <v>656</v>
+        <v>701</v>
       </c>
       <c r="D5" s="6">
         <f>D4-F5</f>
         <v>904</v>
       </c>
       <c r="E5" s="6">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="F5" s="6">
         <v>29</v>
@@ -3880,13 +3915,18 @@
       </c>
       <c r="C6" s="6">
         <f t="shared" si="0"/>
-        <v>525</v>
-      </c>
-      <c r="D6" s="6"/>
+        <v>585</v>
+      </c>
+      <c r="D6" s="6">
+        <f>D5-F6</f>
+        <v>874</v>
+      </c>
       <c r="E6" s="6">
-        <v>131</v>
-      </c>
-      <c r="F6" s="6"/>
+        <v>116</v>
+      </c>
+      <c r="F6" s="6">
+        <v>30</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
@@ -3897,11 +3937,11 @@
       </c>
       <c r="C7" s="6">
         <f t="shared" si="0"/>
-        <v>394</v>
+        <v>469</v>
       </c>
       <c r="D7" s="6"/>
       <c r="E7" s="6">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="F7" s="6"/>
     </row>
@@ -3914,11 +3954,11 @@
       </c>
       <c r="C8" s="6">
         <f t="shared" si="0"/>
-        <v>263</v>
+        <v>353</v>
       </c>
       <c r="D8" s="6"/>
       <c r="E8" s="6">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="F8" s="6"/>
     </row>
@@ -3931,11 +3971,11 @@
       </c>
       <c r="C9" s="6">
         <f t="shared" si="0"/>
-        <v>132</v>
+        <v>237</v>
       </c>
       <c r="D9" s="6"/>
       <c r="E9" s="6">
-        <v>132</v>
+        <v>116</v>
       </c>
       <c r="F9" s="6"/>
     </row>
@@ -3948,11 +3988,30 @@
       </c>
       <c r="C10" s="6">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>121</v>
       </c>
       <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
+      <c r="E10" s="6">
+        <v>116</v>
+      </c>
       <c r="F10" s="6"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" s="5">
+        <v>9</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C11" s="6">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6">
+        <v>121</v>
+      </c>
+      <c r="F11" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3962,7 +4021,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A735EDFD-2DED-4B82-BC46-A3A7E7C548CD}">
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="29.1796875" bestFit="1" customWidth="1"/>
@@ -3974,31 +4033,31 @@
         <v>0</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>27</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
@@ -4006,16 +4065,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="C2" s="1">
-        <v>63</v>
+        <v>27</v>
       </c>
       <c r="D2" s="1">
-        <v>91</v>
+        <v>51</v>
       </c>
       <c r="E2" s="1">
-        <v>87</v>
+        <v>67</v>
+      </c>
+      <c r="F2" s="1">
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
@@ -4023,16 +4085,19 @@
         <v>1</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="C3" s="1">
+        <v>19</v>
+      </c>
+      <c r="D3" s="1">
+        <v>19</v>
+      </c>
+      <c r="E3" s="1">
+        <v>30</v>
+      </c>
+      <c r="F3" s="1">
         <v>0</v>
-      </c>
-      <c r="D3" s="1">
-        <v>0</v>
-      </c>
-      <c r="E3" s="1">
-        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
@@ -4040,16 +4105,19 @@
         <v>1</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="C4" s="1">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4" s="1">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="E4" s="1">
-        <v>46</v>
+        <v>39</v>
+      </c>
+      <c r="F4" s="1">
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
@@ -4057,16 +4125,19 @@
         <v>1</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="C5" s="1">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D5" s="1">
-        <v>16</v>
+        <v>43</v>
       </c>
       <c r="E5" s="1">
-        <v>27</v>
+        <v>51</v>
+      </c>
+      <c r="F5" s="1">
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
@@ -4074,16 +4145,19 @@
         <v>1</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>23</v>
+        <v>44</v>
       </c>
       <c r="C6" s="1">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D6" s="1">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E6" s="1">
-        <v>27</v>
+        <v>21</v>
+      </c>
+      <c r="F6" s="1">
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
@@ -4091,145 +4165,151 @@
         <v>1</v>
       </c>
       <c r="B7" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="1">
+        <v>5</v>
+      </c>
+      <c r="D7" s="1">
+        <v>21</v>
+      </c>
+      <c r="E7" s="1">
         <v>24</v>
       </c>
-      <c r="C7" s="1">
-        <v>16</v>
-      </c>
-      <c r="D7" s="1">
-        <v>30</v>
-      </c>
-      <c r="E7" s="1">
-        <v>38</v>
+      <c r="F7" s="1">
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="1">
         <v>25</v>
       </c>
-      <c r="C8" s="2">
-        <f>SUM(C2:C7)</f>
-        <v>119</v>
-      </c>
-      <c r="D8" s="2">
-        <f t="shared" ref="D8:J8" si="0">SUM(D2:D7)</f>
-        <v>190</v>
-      </c>
-      <c r="E8" s="2">
-        <f t="shared" si="0"/>
-        <v>258</v>
-      </c>
-      <c r="F8" s="2">
+      <c r="D8" s="1">
+        <v>35</v>
+      </c>
+      <c r="E8" s="1">
+        <v>41</v>
+      </c>
+      <c r="F8" s="1">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="2">
+        <f>SUM(C2:C8)</f>
+        <v>116</v>
+      </c>
+      <c r="D9" s="2">
+        <f>SUM(D2:D8)</f>
+        <v>213</v>
+      </c>
+      <c r="E9" s="2">
+        <f>SUM(E2:E8)</f>
+        <v>273</v>
+      </c>
+      <c r="F9" s="2">
+        <f>SUM(F2:F8)</f>
+        <v>321</v>
+      </c>
+      <c r="G9" s="2">
+        <f t="shared" ref="G9:J9" si="0">SUM(G3:G8)</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G8" s="2">
+      <c r="I9" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="2">
+      <c r="J9" s="2">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I8" s="2">
-        <f t="shared" si="0"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="2">
+        <f>SUM(C2:C8)-C8</f>
+        <v>91</v>
+      </c>
+      <c r="D10" s="2">
+        <f>SUM(D2:D8)-D8</f>
+        <v>178</v>
+      </c>
+      <c r="E10" s="2">
+        <f>SUM(E2:E8)-E8</f>
+        <v>232</v>
+      </c>
+      <c r="F10" s="2">
+        <f>SUM(F2:F8)-F8</f>
+        <v>246</v>
+      </c>
+      <c r="G10" s="2">
+        <f t="shared" ref="G10:J10" si="1">SUM(G3:G8)-G8</f>
         <v>0</v>
       </c>
-      <c r="J8" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>1</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="C9" s="2">
-        <f>SUM(C2:C7)-C7</f>
-        <v>103</v>
-      </c>
-      <c r="D9" s="2">
-        <f t="shared" ref="D9:J9" si="1">SUM(D2:D7)-D7</f>
-        <v>160</v>
-      </c>
-      <c r="E9" s="2">
-        <f>SUM(E2:E7)-E7</f>
-        <v>220</v>
-      </c>
-      <c r="F9" s="2">
+      <c r="H10" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G9" s="2">
+      <c r="I10" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H9" s="2">
+      <c r="J10" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I9" s="2">
-        <f t="shared" si="1"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A12" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="J9" s="2">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A11" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" s="2" t="s">
+      <c r="B12" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="I12" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="J12" s="2" t="s">
         <v>27</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>1</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="C12" s="1">
-        <v>23</v>
-      </c>
-      <c r="D12" s="1">
-        <v>23</v>
-      </c>
-      <c r="E12" s="1">
-        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
@@ -4237,16 +4317,19 @@
         <v>1</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="C13" s="1">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="D13" s="1">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="E13" s="1">
-        <v>5</v>
+        <v>41</v>
+      </c>
+      <c r="F13" s="1">
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
@@ -4254,16 +4337,19 @@
         <v>1</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="C14" s="1">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="D14" s="1">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="E14" s="1">
-        <v>16</v>
+        <v>6</v>
+      </c>
+      <c r="F14" s="1">
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
@@ -4271,16 +4357,19 @@
         <v>1</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="C15" s="1">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="D15" s="1">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="E15" s="1">
-        <v>12</v>
+        <v>19</v>
+      </c>
+      <c r="F15" s="1">
+        <v>25</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
@@ -4288,16 +4377,19 @@
         <v>1</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C16" s="1">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="D16" s="1">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E16" s="1">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="F16" s="1">
+        <v>14</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
@@ -4305,16 +4397,19 @@
         <v>1</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="C17" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D17" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E17" s="1">
-        <v>18</v>
+        <v>9</v>
+      </c>
+      <c r="F17" s="1">
+        <v>8</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
@@ -4322,16 +4417,19 @@
         <v>1</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="C18" s="1">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D18" s="1">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="E18" s="1">
-        <v>4</v>
+        <v>26</v>
+      </c>
+      <c r="F18" s="1">
+        <v>37</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
@@ -4339,16 +4437,19 @@
         <v>1</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="C19" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D19" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E19" s="1">
-        <v>7</v>
+        <v>2</v>
+      </c>
+      <c r="F19" s="1">
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
@@ -4356,16 +4457,19 @@
         <v>1</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="C20" s="1">
         <v>0</v>
       </c>
       <c r="D20" s="1">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E20" s="1">
-        <v>23</v>
+        <v>8</v>
+      </c>
+      <c r="F20" s="1">
+        <v>8</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
@@ -4373,16 +4477,19 @@
         <v>1</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="C21" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D21" s="1">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="E21" s="1">
-        <v>16</v>
+        <v>23</v>
+      </c>
+      <c r="F21" s="1">
+        <v>23</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.35">
@@ -4390,16 +4497,19 @@
         <v>1</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="C22" s="1">
         <v>0</v>
       </c>
       <c r="D22" s="1">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E22" s="1">
-        <v>32</v>
+        <v>19</v>
+      </c>
+      <c r="F22" s="1">
+        <v>25</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
@@ -4407,16 +4517,19 @@
         <v>1</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="C23" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D23" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E23" s="1">
-        <v>10</v>
+        <v>35</v>
+      </c>
+      <c r="F23" s="1">
+        <v>38</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.35">
@@ -4427,13 +4540,16 @@
         <v>41</v>
       </c>
       <c r="C24" s="1">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="D24" s="1">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="E24" s="1">
-        <v>37</v>
+        <v>9</v>
+      </c>
+      <c r="F24" s="1">
+        <v>9</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
@@ -4441,56 +4557,39 @@
         <v>1</v>
       </c>
       <c r="B25" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C25" s="1">
+        <v>5</v>
+      </c>
+      <c r="D25" s="1">
+        <v>21</v>
+      </c>
+      <c r="E25" s="1">
         <v>24</v>
       </c>
-      <c r="C25" s="1">
-        <v>16</v>
-      </c>
-      <c r="D25" s="1">
-        <v>30</v>
-      </c>
-      <c r="E25" s="1">
-        <v>38</v>
+      <c r="F25" s="1">
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>1</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="B26" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26" s="1">
         <v>25</v>
       </c>
-      <c r="C26" s="2">
-        <f>SUM(C12:C25)</f>
-        <v>119</v>
-      </c>
-      <c r="D26" s="2">
-        <f>SUM(D12:D25)</f>
-        <v>190</v>
-      </c>
-      <c r="E26" s="2">
-        <f>SUM(E12:E25)</f>
-        <v>258</v>
-      </c>
-      <c r="F26" s="2">
-        <f t="shared" ref="F26" si="2">SUM(F15:F24)</f>
-        <v>0</v>
-      </c>
-      <c r="G26" s="2">
-        <f t="shared" ref="G26" si="3">SUM(G15:G24)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="2">
-        <f t="shared" ref="H26" si="4">SUM(H15:H24)</f>
-        <v>0</v>
-      </c>
-      <c r="I26" s="2">
-        <f t="shared" ref="I26" si="5">SUM(I15:I24)</f>
-        <v>0</v>
-      </c>
-      <c r="J26" s="2">
-        <f t="shared" ref="J26" si="6">SUM(J15:J24)</f>
-        <v>0</v>
+      <c r="D26" s="1">
+        <v>35</v>
+      </c>
+      <c r="E26" s="1">
+        <v>41</v>
+      </c>
+      <c r="F26" s="1">
+        <v>75</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.35">
@@ -4498,38 +4597,78 @@
         <v>1</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="C27" s="2">
-        <f>SUM(C12:C25)-C25</f>
-        <v>103</v>
+        <f>SUM(C13:C26)</f>
+        <v>116</v>
       </c>
       <c r="D27" s="2">
-        <f>SUM(D12:D25)-D25</f>
-        <v>160</v>
+        <f>SUM(D13:D26)</f>
+        <v>213</v>
       </c>
       <c r="E27" s="2">
-        <f>SUM(E12:E25)-E25</f>
-        <v>220</v>
+        <f>SUM(E13:E26)</f>
+        <v>273</v>
       </c>
       <c r="F27" s="2">
-        <f t="shared" ref="E27:J27" si="7">SUM(F15:F24)-F24</f>
+        <f>SUM(F13:F26)</f>
+        <v>321</v>
+      </c>
+      <c r="G27" s="2">
+        <f t="shared" ref="G27:J27" si="2">SUM(G13:G26)</f>
         <v>0</v>
       </c>
-      <c r="G27" s="2">
-        <f t="shared" si="7"/>
+      <c r="H27" s="2">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="H27" s="2">
-        <f t="shared" si="7"/>
+      <c r="I27" s="2">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="I27" s="2">
-        <f t="shared" si="7"/>
+      <c r="J27" s="2">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J27" s="2">
-        <f t="shared" si="7"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>1</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C28" s="2">
+        <f>SUM(C13:C26)-C26</f>
+        <v>91</v>
+      </c>
+      <c r="D28" s="2">
+        <f>SUM(D13:D26)-D26</f>
+        <v>178</v>
+      </c>
+      <c r="E28" s="2">
+        <f>SUM(E13:E26)-E26</f>
+        <v>232</v>
+      </c>
+      <c r="F28" s="2">
+        <f>SUM(F13:F26)-F26</f>
+        <v>246</v>
+      </c>
+      <c r="G28" s="2">
+        <f t="shared" ref="G28:J28" si="3">SUM(G13:G26)-G26</f>
+        <v>0</v>
+      </c>
+      <c r="H28" s="2">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="I28" s="2">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J28" s="2">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: parser Obs_1/Obs_2 flexible, filtro app en 3 hojas, ocultar valores 0 en obs, burndown solo funcionalidades, grafico centrado y compacto
</commit_message>
<xml_diff>
--- a/Presentación Semanal UAT.xlsx
+++ b/Presentación Semanal UAT.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\QA\WrampUp - copia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E571F51-14C2-4EAF-A1A6-1D6523B036B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A7EC188-9DBA-45C5-9F51-38445C80005F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{27A98AC9-9505-493B-985E-2D79FFCBCA40}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{27A98AC9-9505-493B-985E-2D79FFCBCA40}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="1" r:id="rId1"/>
     <sheet name="BC_F" sheetId="3" r:id="rId2"/>
     <sheet name="BC_CP" sheetId="2" r:id="rId3"/>
-    <sheet name="Obs" sheetId="4" r:id="rId4"/>
+    <sheet name="Obs_1" sheetId="4" r:id="rId4"/>
+    <sheet name="Obs_2" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="52">
   <si>
     <t>Aplicación</t>
   </si>
@@ -170,9 +171,6 @@
     <t>Simulación de Préstamos</t>
   </si>
   <si>
-    <t>ISSUE</t>
-  </si>
-  <si>
     <t>DEFECTO FUNCIONAL</t>
   </si>
   <si>
@@ -190,12 +188,24 @@
   <si>
     <t>ODS SPACE - Reclamos y Dalis</t>
   </si>
+  <si>
+    <t>Registro del Reclamo</t>
+  </si>
+  <si>
+    <t>Consulta del Reclamo</t>
+  </si>
+  <si>
+    <t>ISSUE - CRÍTICO</t>
+  </si>
+  <si>
+    <t>ISSUE - NO CRÍTICO</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -225,6 +235,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -246,7 +265,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -269,16 +288,93 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -292,14 +388,61 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -439,22 +582,22 @@
                   <c:v>156</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>133</c:v>
+                  <c:v>136</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>110</c:v>
+                  <c:v>116</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>87</c:v>
+                  <c:v>93</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>64</c:v>
+                  <c:v>70</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>41</c:v>
+                  <c:v>47</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>18</c:v>
+                  <c:v>24</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -650,6 +793,9 @@
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>116</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>86</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1127,6 +1273,9 @@
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>874</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>829</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3446,106 +3595,106 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="11">
+      <c r="A2" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8">
         <v>328</v>
       </c>
-      <c r="C2" s="6">
+      <c r="C2" s="5">
         <v>202</v>
       </c>
-      <c r="D2" s="7">
+      <c r="D2" s="6">
         <f>(C2*100)/B2</f>
         <v>61.585365853658537</v>
       </c>
-      <c r="E2" s="6">
+      <c r="E2" s="5">
         <v>1049</v>
       </c>
-      <c r="F2" s="6" t="s">
-        <v>47</v>
+      <c r="F2" s="5" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="11">
+      <c r="B3" s="8">
         <v>46</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3" s="5">
         <v>5</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="6">
         <f>(C3*100)/B3</f>
         <v>10.869565217391305</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="5">
         <v>74</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="8">
         <v>82</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="5">
         <v>7</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D4" s="6">
         <f t="shared" ref="D4:D5" si="0">(C4*100)/B4</f>
         <v>8.536585365853659</v>
       </c>
-      <c r="E4" s="6">
-        <v>161</v>
-      </c>
-      <c r="F4" s="6" t="s">
+      <c r="E4" s="5">
+        <v>154</v>
+      </c>
+      <c r="F4" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="B5" s="11">
+      <c r="A5" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5" s="8">
         <v>37</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="5">
         <v>8</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="6">
         <f t="shared" si="0"/>
         <v>21.621621621621621</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="5">
         <v>47</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="5" t="s">
         <v>9</v>
       </c>
     </row>
@@ -3557,11 +3706,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42DF1849-A1A9-4E05-97A1-E2B79B421503}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.36328125" style="1" customWidth="1"/>
     <col min="5" max="5" width="18" style="1" bestFit="1" customWidth="1"/>
@@ -3569,217 +3718,279 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="12">
+      <c r="A2" s="9">
         <v>0</v>
       </c>
-      <c r="B2" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="13">
+      <c r="B2" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="10">
         <v>202</v>
       </c>
-      <c r="D2" s="13">
+      <c r="D2" s="10">
         <v>202</v>
       </c>
-      <c r="E2" s="13">
+      <c r="E2" s="10">
         <v>23</v>
       </c>
-      <c r="F2" s="13">
+      <c r="F2" s="10">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="5">
-        <v>1</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="6">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="5">
         <f>C2-$E$2</f>
         <v>179</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="5">
         <f>D2-F3</f>
         <v>164</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="5">
         <v>23</v>
       </c>
-      <c r="F3" s="6">
+      <c r="F3" s="5">
         <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="5">
+      <c r="A4" s="4">
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="6">
+      <c r="B4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="5">
         <f>C3-$E$2</f>
         <v>156</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="5">
         <f>D3-F4</f>
         <v>144</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="5">
         <v>23</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="5">
         <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="5">
+      <c r="A5" s="4">
         <v>3</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C5" s="6">
-        <f t="shared" ref="C5:C11" si="0">C4-$E$2</f>
-        <v>133</v>
-      </c>
-      <c r="D5" s="6">
+      <c r="B5" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="5">
+        <f>C4-20</f>
+        <v>136</v>
+      </c>
+      <c r="D5" s="5">
         <f>D4-F5</f>
         <v>129</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="5">
         <v>20</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="5">
         <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="5">
+      <c r="A6" s="4">
         <v>4</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" s="6">
-        <f t="shared" si="0"/>
-        <v>110</v>
-      </c>
-      <c r="D6" s="6">
+      <c r="B6" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="5">
+        <f>C5-20</f>
+        <v>116</v>
+      </c>
+      <c r="D6" s="5">
         <f>D5-F6</f>
         <v>116</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="5">
         <v>20</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="5">
         <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" s="5">
+      <c r="A7" s="4">
         <v>5</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C7" s="6">
+      <c r="B7" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="5">
+        <f>C6-$E$2</f>
+        <v>93</v>
+      </c>
+      <c r="D7" s="5">
+        <f>D6-F7</f>
+        <v>86</v>
+      </c>
+      <c r="E7" s="5">
+        <v>23</v>
+      </c>
+      <c r="F7" s="5">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" s="4">
+        <v>6</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" s="5">
+        <f t="shared" ref="C5:C11" si="0">C7-$E$2</f>
+        <v>70</v>
+      </c>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5">
+        <v>23</v>
+      </c>
+      <c r="F8" s="5"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" s="4">
+        <v>7</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" s="5">
         <f t="shared" si="0"/>
-        <v>87</v>
-      </c>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6">
+        <v>47</v>
+      </c>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5">
         <v>23</v>
       </c>
-      <c r="F7" s="6"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8" s="5">
+      <c r="F9" s="5"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" s="4">
+        <v>8</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" s="5">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5">
+        <v>23</v>
+      </c>
+      <c r="F10" s="5"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" s="4">
+        <v>9</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C11" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5">
+        <v>24</v>
+      </c>
+      <c r="F11" s="5"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" s="4">
+        <v>0</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" s="5">
+        <v>8</v>
+      </c>
+      <c r="D12" s="5">
+        <v>8</v>
+      </c>
+      <c r="E12" s="5">
+        <v>4</v>
+      </c>
+      <c r="F12" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" s="4">
+        <v>1</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C13" s="5">
+        <v>4</v>
+      </c>
+      <c r="D13" s="5">
+        <f>D12-F13</f>
+        <v>2</v>
+      </c>
+      <c r="E13" s="5">
+        <v>4</v>
+      </c>
+      <c r="F13" s="5">
         <v>6</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C8" s="6">
-        <f t="shared" si="0"/>
-        <v>64</v>
-      </c>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6">
-        <v>23</v>
-      </c>
-      <c r="F8" s="6"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9" s="5">
-        <v>7</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C9" s="6">
-        <f t="shared" si="0"/>
-        <v>41</v>
-      </c>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6">
-        <v>23</v>
-      </c>
-      <c r="F9" s="6"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10" s="5">
-        <v>8</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C10" s="6">
-        <f t="shared" si="0"/>
-        <v>18</v>
-      </c>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6">
-        <v>23</v>
-      </c>
-      <c r="F10" s="6"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" s="5">
-        <v>9</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C11" s="6">
-        <f t="shared" si="0"/>
-        <v>-5</v>
-      </c>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6">
-        <v>24</v>
-      </c>
-      <c r="F11" s="6"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" s="4">
+        <v>2</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="5">
+        <v>4</v>
+      </c>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5">
+        <v>4</v>
+      </c>
+      <c r="F14" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3789,11 +4000,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20BCB52B-56FF-4E38-A246-A8F336FD8B79}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.36328125" style="1" customWidth="1"/>
     <col min="5" max="5" width="18" style="1" bestFit="1" customWidth="1"/>
@@ -3801,217 +4012,279 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="12">
+      <c r="A2" s="9">
         <v>0</v>
       </c>
-      <c r="B2" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="13">
+      <c r="B2" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="10">
         <v>1049</v>
       </c>
-      <c r="D2" s="13">
+      <c r="D2" s="10">
         <v>1049</v>
       </c>
-      <c r="E2" s="13">
+      <c r="E2" s="10">
         <v>116</v>
       </c>
-      <c r="F2" s="13">
+      <c r="F2" s="10">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="5">
-        <v>1</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="6">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="5">
         <f>C2-$E$2</f>
         <v>933</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="5">
         <f>D2-F3</f>
         <v>983</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="5">
         <v>116</v>
       </c>
-      <c r="F3" s="6">
+      <c r="F3" s="5">
         <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="5">
+      <c r="A4" s="4">
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="6">
+      <c r="B4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="5">
         <f t="shared" ref="C4:C11" si="0">C3-$E$2</f>
         <v>817</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="5">
         <f>D3-F4</f>
         <v>933</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="5">
         <v>116</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="5">
         <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="5">
+      <c r="A5" s="4">
         <v>3</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C5" s="6">
+      <c r="B5" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="5">
         <f t="shared" si="0"/>
         <v>701</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="5">
         <f>D4-F5</f>
         <v>904</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="5">
         <v>116</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="5">
         <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="5">
+      <c r="A6" s="4">
         <v>4</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" s="6">
+      <c r="B6" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="5">
         <f t="shared" si="0"/>
         <v>585</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="5">
         <f>D5-F6</f>
         <v>874</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="5">
         <v>116</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="5">
         <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" s="5">
+      <c r="A7" s="4">
         <v>5</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C7" s="6">
+      <c r="B7" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="5">
         <f t="shared" si="0"/>
         <v>469</v>
       </c>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6">
+      <c r="D7" s="5">
+        <f>D6-F7</f>
+        <v>829</v>
+      </c>
+      <c r="E7" s="5">
         <v>116</v>
       </c>
-      <c r="F7" s="6"/>
+      <c r="F7" s="5">
+        <v>45</v>
+      </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8" s="5">
+      <c r="A8" s="4">
         <v>6</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C8" s="6">
+      <c r="B8" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" s="5">
         <f t="shared" si="0"/>
         <v>353</v>
       </c>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6">
+      <c r="D8" s="5"/>
+      <c r="E8" s="5">
         <v>116</v>
       </c>
-      <c r="F8" s="6"/>
+      <c r="F8" s="5"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9" s="5">
+      <c r="A9" s="4">
         <v>7</v>
       </c>
-      <c r="B9" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C9" s="6">
+      <c r="B9" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" s="5">
         <f t="shared" si="0"/>
         <v>237</v>
       </c>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6">
+      <c r="D9" s="5"/>
+      <c r="E9" s="5">
         <v>116</v>
       </c>
-      <c r="F9" s="6"/>
+      <c r="F9" s="5"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10" s="5">
+      <c r="A10" s="4">
         <v>8</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C10" s="6">
+      <c r="B10" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" s="5">
         <f t="shared" si="0"/>
         <v>121</v>
       </c>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6">
+      <c r="D10" s="5"/>
+      <c r="E10" s="5">
         <v>116</v>
       </c>
-      <c r="F10" s="6"/>
+      <c r="F10" s="5"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" s="5">
+      <c r="A11" s="4">
         <v>9</v>
       </c>
-      <c r="B11" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C11" s="6">
+      <c r="B11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C11" s="5">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6">
+      <c r="D11" s="5"/>
+      <c r="E11" s="5">
         <v>121</v>
       </c>
-      <c r="F11" s="6"/>
+      <c r="F11" s="5"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" s="4">
+        <v>0</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" s="5">
+        <v>47</v>
+      </c>
+      <c r="D12" s="5">
+        <v>47</v>
+      </c>
+      <c r="E12" s="5">
+        <v>32</v>
+      </c>
+      <c r="F12" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" s="4">
+        <v>1</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C13" s="5">
+        <v>23</v>
+      </c>
+      <c r="D13" s="5">
+        <f>D12-F13</f>
+        <v>11</v>
+      </c>
+      <c r="E13" s="5">
+        <v>32</v>
+      </c>
+      <c r="F13" s="5">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" s="4">
+        <v>2</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="5">
+        <v>24</v>
+      </c>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5">
+        <v>15</v>
+      </c>
+      <c r="F14" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4021,51 +4294,52 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A735EDFD-2DED-4B82-BC46-A3A7E7C548CD}">
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="1" max="1" width="25.453125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29.1796875" bestFit="1" customWidth="1"/>
     <col min="3" max="10" width="10.90625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="14" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>42</v>
+      <c r="A2" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>50</v>
       </c>
       <c r="C2" s="1">
         <v>27</v>
@@ -4079,596 +4353,705 @@
       <c r="F2" s="1">
         <v>79</v>
       </c>
+      <c r="G2" s="1">
+        <v>12</v>
+      </c>
+      <c r="J2" s="17"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>17</v>
+      <c r="A3" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>51</v>
       </c>
       <c r="C3" s="1">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="D3" s="1">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="E3" s="1">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F3" s="1">
         <v>0</v>
       </c>
+      <c r="G3" s="1">
+        <v>81</v>
+      </c>
+      <c r="J3" s="17"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>46</v>
+      <c r="A4" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>17</v>
       </c>
       <c r="C4" s="1">
+        <v>19</v>
+      </c>
+      <c r="D4" s="1">
+        <v>19</v>
+      </c>
+      <c r="E4" s="1">
+        <v>30</v>
+      </c>
+      <c r="F4" s="1">
+        <v>0</v>
+      </c>
+      <c r="G4" s="1">
+        <v>13</v>
+      </c>
+      <c r="J4" s="17"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A5" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" s="1">
         <v>16</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D5" s="1">
         <v>29</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E5" s="1">
         <v>39</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F5" s="1">
         <v>45</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" s="8" t="s">
+      <c r="G5" s="1">
+        <v>45</v>
+      </c>
+      <c r="J5" s="17"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A6" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" s="1">
+        <v>11</v>
+      </c>
+      <c r="D6" s="1">
         <v>43</v>
       </c>
-      <c r="C5" s="1">
+      <c r="E6" s="1">
+        <v>51</v>
+      </c>
+      <c r="F6" s="1">
+        <v>93</v>
+      </c>
+      <c r="G6" s="1">
+        <v>85</v>
+      </c>
+      <c r="J6" s="17"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A7" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" s="1">
+        <v>13</v>
+      </c>
+      <c r="D7" s="1">
+        <v>15</v>
+      </c>
+      <c r="E7" s="1">
+        <v>21</v>
+      </c>
+      <c r="F7" s="1">
+        <v>21</v>
+      </c>
+      <c r="G7" s="1">
+        <v>0</v>
+      </c>
+      <c r="J7" s="17"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" s="1">
+        <v>5</v>
+      </c>
+      <c r="D8" s="1">
+        <v>21</v>
+      </c>
+      <c r="E8" s="1">
+        <v>24</v>
+      </c>
+      <c r="F8" s="1">
+        <v>8</v>
+      </c>
+      <c r="G8" s="1">
+        <v>0</v>
+      </c>
+      <c r="J8" s="17"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="1">
+        <v>25</v>
+      </c>
+      <c r="D9" s="1">
+        <v>35</v>
+      </c>
+      <c r="E9" s="1">
+        <v>41</v>
+      </c>
+      <c r="F9" s="1">
+        <v>75</v>
+      </c>
+      <c r="G9" s="1">
+        <v>101</v>
+      </c>
+      <c r="J9" s="17"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="19">
+        <f>SUM(C2:C9)</f>
+        <v>116</v>
+      </c>
+      <c r="D10" s="19">
+        <f>SUM(D2:D9)</f>
+        <v>213</v>
+      </c>
+      <c r="E10" s="19">
+        <f>SUM(E2:E9)</f>
+        <v>273</v>
+      </c>
+      <c r="F10" s="19">
+        <f>SUM(F2:F9)</f>
+        <v>321</v>
+      </c>
+      <c r="G10" s="19">
+        <f>SUM(G2:G9)</f>
+        <v>337</v>
+      </c>
+      <c r="H10" s="19">
+        <f>SUM(H4:H9)</f>
+        <v>0</v>
+      </c>
+      <c r="I10" s="19">
+        <f>SUM(I4:I9)</f>
+        <v>0</v>
+      </c>
+      <c r="J10" s="20">
+        <f>SUM(J4:J9)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" s="19">
+        <f>SUM(C2:C9)-C9</f>
+        <v>91</v>
+      </c>
+      <c r="D11" s="19">
+        <f>SUM(D2:D9)-D9</f>
+        <v>178</v>
+      </c>
+      <c r="E11" s="19">
+        <f>SUM(E2:E9)-E9</f>
+        <v>232</v>
+      </c>
+      <c r="F11" s="19">
+        <f>SUM(F2:F9)-F9</f>
+        <v>246</v>
+      </c>
+      <c r="G11" s="19">
+        <f>SUM(G2:G9)-G9</f>
+        <v>236</v>
+      </c>
+      <c r="H11" s="19">
+        <f>SUM(H4:H9)-H9</f>
+        <v>0</v>
+      </c>
+      <c r="I11" s="19">
+        <f>SUM(I4:I9)-I9</f>
+        <v>0</v>
+      </c>
+      <c r="J11" s="20">
+        <f>SUM(J4:J9)-J9</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A13" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="G13" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="H13" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="I13" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="J13" s="14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A14" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="1">
+        <v>38</v>
+      </c>
+      <c r="D14" s="1">
+        <v>38</v>
+      </c>
+      <c r="E14" s="1">
+        <v>41</v>
+      </c>
+      <c r="F14" s="1">
+        <v>48</v>
+      </c>
+      <c r="G14" s="1">
+        <v>49</v>
+      </c>
+      <c r="J14" s="17"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A15" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" s="1">
+        <v>6</v>
+      </c>
+      <c r="D15" s="1">
+        <v>6</v>
+      </c>
+      <c r="E15" s="1">
+        <v>6</v>
+      </c>
+      <c r="F15" s="1">
+        <v>9</v>
+      </c>
+      <c r="G15" s="1">
+        <v>9</v>
+      </c>
+      <c r="J15" s="17"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A16" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16" s="1">
+        <v>15</v>
+      </c>
+      <c r="D16" s="1">
+        <v>19</v>
+      </c>
+      <c r="E16" s="1">
+        <v>19</v>
+      </c>
+      <c r="F16" s="1">
+        <v>25</v>
+      </c>
+      <c r="G16" s="1">
+        <v>23</v>
+      </c>
+      <c r="J16" s="17"/>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A17" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B17" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" s="1">
         <v>11</v>
       </c>
-      <c r="D5" s="1">
-        <v>43</v>
-      </c>
-      <c r="E5" s="1">
-        <v>51</v>
-      </c>
-      <c r="F5" s="1">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B6" s="8" t="s">
+      <c r="D17" s="1">
+        <v>11</v>
+      </c>
+      <c r="E17" s="1">
+        <v>11</v>
+      </c>
+      <c r="F17" s="1">
+        <v>14</v>
+      </c>
+      <c r="G17" s="1">
+        <v>14</v>
+      </c>
+      <c r="J17" s="17"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A18" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B18" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="C18" s="1">
+        <v>5</v>
+      </c>
+      <c r="D18" s="1">
+        <v>9</v>
+      </c>
+      <c r="E18" s="1">
+        <v>9</v>
+      </c>
+      <c r="F18" s="1">
+        <v>8</v>
+      </c>
+      <c r="G18" s="1">
+        <v>8</v>
+      </c>
+      <c r="J18" s="17"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A19" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B19" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" s="1">
+        <v>8</v>
+      </c>
+      <c r="D19" s="1">
+        <v>25</v>
+      </c>
+      <c r="E19" s="1">
+        <v>26</v>
+      </c>
+      <c r="F19" s="1">
+        <v>37</v>
+      </c>
+      <c r="G19" s="1">
+        <v>34</v>
+      </c>
+      <c r="J19" s="17"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A20" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="C20" s="1">
+        <v>1</v>
+      </c>
+      <c r="D20" s="1">
+        <v>2</v>
+      </c>
+      <c r="E20" s="1">
+        <v>2</v>
+      </c>
+      <c r="F20" s="1">
+        <v>2</v>
+      </c>
+      <c r="G20" s="1">
+        <v>2</v>
+      </c>
+      <c r="J20" s="17"/>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A21" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B21" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" s="1">
+        <v>0</v>
+      </c>
+      <c r="D21" s="1">
+        <v>6</v>
+      </c>
+      <c r="E21" s="1">
+        <v>8</v>
+      </c>
+      <c r="F21" s="1">
+        <v>8</v>
+      </c>
+      <c r="G21" s="1">
+        <v>3</v>
+      </c>
+      <c r="J21" s="17"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A22" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B22" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="C22" s="1">
+        <v>1</v>
+      </c>
+      <c r="D22" s="1">
+        <v>18</v>
+      </c>
+      <c r="E22" s="1">
+        <v>23</v>
+      </c>
+      <c r="F22" s="1">
+        <v>23</v>
+      </c>
+      <c r="G22" s="1">
+        <v>26</v>
+      </c>
+      <c r="J22" s="17"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A23" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="C23" s="1">
+        <v>0</v>
+      </c>
+      <c r="D23" s="1">
+        <v>19</v>
+      </c>
+      <c r="E23" s="1">
+        <v>19</v>
+      </c>
+      <c r="F23" s="1">
+        <v>25</v>
+      </c>
+      <c r="G23" s="1">
+        <v>21</v>
+      </c>
+      <c r="J23" s="17"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A24" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B24" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="C24" s="1">
+        <v>1</v>
+      </c>
+      <c r="D24" s="1">
+        <v>4</v>
+      </c>
+      <c r="E24" s="1">
+        <v>35</v>
+      </c>
+      <c r="F24" s="1">
+        <v>38</v>
+      </c>
+      <c r="G24" s="1">
+        <v>38</v>
+      </c>
+      <c r="J24" s="17"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A25" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B25" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C25" s="1">
+        <v>0</v>
+      </c>
+      <c r="D25" s="1">
+        <v>0</v>
+      </c>
+      <c r="E25" s="1">
+        <v>9</v>
+      </c>
+      <c r="F25" s="1">
+        <v>9</v>
+      </c>
+      <c r="G25" s="1">
+        <v>9</v>
+      </c>
+      <c r="J25" s="17"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A26" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B26" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="C6" s="1">
-        <v>13</v>
-      </c>
-      <c r="D6" s="1">
-        <v>15</v>
-      </c>
-      <c r="E6" s="1">
+      <c r="C26" s="1">
+        <v>5</v>
+      </c>
+      <c r="D26" s="1">
         <v>21</v>
       </c>
-      <c r="F6" s="1">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="C7" s="1">
-        <v>5</v>
-      </c>
-      <c r="D7" s="1">
-        <v>21</v>
-      </c>
-      <c r="E7" s="1">
+      <c r="E26" s="1">
         <v>24</v>
       </c>
-      <c r="F7" s="1">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>1</v>
-      </c>
-      <c r="B8" s="8" t="s">
+      <c r="F26" s="1">
+        <v>0</v>
+      </c>
+      <c r="G26" s="1">
+        <v>0</v>
+      </c>
+      <c r="J26" s="17"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A27" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B27" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C27" s="1">
         <v>25</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D27" s="1">
         <v>35</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E27" s="1">
         <v>41</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F27" s="1">
         <v>75</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>1</v>
-      </c>
-      <c r="B9" s="9" t="s">
+      <c r="G27" s="1">
+        <v>101</v>
+      </c>
+      <c r="J27" s="17"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A28" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B28" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="2">
-        <f>SUM(C2:C8)</f>
+      <c r="C28" s="19">
+        <f t="shared" ref="C28:J28" si="0">SUM(C14:C27)</f>
         <v>116</v>
       </c>
-      <c r="D9" s="2">
-        <f>SUM(D2:D8)</f>
+      <c r="D28" s="19">
+        <f t="shared" si="0"/>
         <v>213</v>
       </c>
-      <c r="E9" s="2">
-        <f>SUM(E2:E8)</f>
+      <c r="E28" s="19">
+        <f t="shared" si="0"/>
         <v>273</v>
       </c>
-      <c r="F9" s="2">
-        <f>SUM(F2:F8)</f>
+      <c r="F28" s="19">
+        <f t="shared" si="0"/>
         <v>321</v>
       </c>
-      <c r="G9" s="2">
-        <f t="shared" ref="G9:J9" si="0">SUM(G3:G8)</f>
-        <v>0</v>
-      </c>
-      <c r="H9" s="2">
+      <c r="G28" s="19">
+        <f t="shared" si="0"/>
+        <v>337</v>
+      </c>
+      <c r="H28" s="19">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I28" s="19">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J28" s="20">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>1</v>
-      </c>
-      <c r="B10" s="9" t="s">
+    <row r="29" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A29" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="B29" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="2">
-        <f>SUM(C2:C8)-C8</f>
+      <c r="C29" s="23">
+        <f t="shared" ref="C29:J29" si="1">SUM(C14:C27)-C27</f>
         <v>91</v>
       </c>
-      <c r="D10" s="2">
-        <f>SUM(D2:D8)-D8</f>
+      <c r="D29" s="23">
+        <f t="shared" si="1"/>
         <v>178</v>
       </c>
-      <c r="E10" s="2">
-        <f>SUM(E2:E8)-E8</f>
+      <c r="E29" s="23">
+        <f t="shared" si="1"/>
         <v>232</v>
       </c>
-      <c r="F10" s="2">
-        <f>SUM(F2:F8)-F8</f>
+      <c r="F29" s="23">
+        <f t="shared" si="1"/>
         <v>246</v>
       </c>
-      <c r="G10" s="2">
-        <f t="shared" ref="G10:J10" si="1">SUM(G3:G8)-G8</f>
-        <v>0</v>
-      </c>
-      <c r="H10" s="2">
+      <c r="G29" s="23">
+        <f t="shared" si="1"/>
+        <v>236</v>
+      </c>
+      <c r="H29" s="23">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I29" s="23">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J29" s="24">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A12" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>1</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C13" s="1">
-        <v>38</v>
-      </c>
-      <c r="D13" s="1">
-        <v>38</v>
-      </c>
-      <c r="E13" s="1">
-        <v>41</v>
-      </c>
-      <c r="F13" s="1">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>1</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C14" s="1">
-        <v>6</v>
-      </c>
-      <c r="D14" s="1">
-        <v>6</v>
-      </c>
-      <c r="E14" s="1">
-        <v>6</v>
-      </c>
-      <c r="F14" s="1">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>1</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="C15" s="1">
-        <v>15</v>
-      </c>
-      <c r="D15" s="1">
-        <v>19</v>
-      </c>
-      <c r="E15" s="1">
-        <v>19</v>
-      </c>
-      <c r="F15" s="1">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>1</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="C16" s="1">
-        <v>11</v>
-      </c>
-      <c r="D16" s="1">
-        <v>11</v>
-      </c>
-      <c r="E16" s="1">
-        <v>11</v>
-      </c>
-      <c r="F16" s="1">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>1</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C17" s="1">
-        <v>5</v>
-      </c>
-      <c r="D17" s="1">
-        <v>9</v>
-      </c>
-      <c r="E17" s="1">
-        <v>9</v>
-      </c>
-      <c r="F17" s="1">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>1</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C18" s="1">
-        <v>8</v>
-      </c>
-      <c r="D18" s="1">
-        <v>25</v>
-      </c>
-      <c r="E18" s="1">
-        <v>26</v>
-      </c>
-      <c r="F18" s="1">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>1</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C19" s="1">
-        <v>1</v>
-      </c>
-      <c r="D19" s="1">
-        <v>2</v>
-      </c>
-      <c r="E19" s="1">
-        <v>2</v>
-      </c>
-      <c r="F19" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>1</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="C20" s="1">
-        <v>0</v>
-      </c>
-      <c r="D20" s="1">
-        <v>6</v>
-      </c>
-      <c r="E20" s="1">
-        <v>8</v>
-      </c>
-      <c r="F20" s="1">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>1</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C21" s="1">
-        <v>1</v>
-      </c>
-      <c r="D21" s="1">
-        <v>18</v>
-      </c>
-      <c r="E21" s="1">
-        <v>23</v>
-      </c>
-      <c r="F21" s="1">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>1</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="C22" s="1">
-        <v>0</v>
-      </c>
-      <c r="D22" s="1">
-        <v>19</v>
-      </c>
-      <c r="E22" s="1">
-        <v>19</v>
-      </c>
-      <c r="F22" s="1">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>1</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C23" s="1">
-        <v>1</v>
-      </c>
-      <c r="D23" s="1">
-        <v>4</v>
-      </c>
-      <c r="E23" s="1">
-        <v>35</v>
-      </c>
-      <c r="F23" s="1">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>1</v>
-      </c>
-      <c r="B24" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="C24" s="1">
-        <v>0</v>
-      </c>
-      <c r="D24" s="1">
-        <v>0</v>
-      </c>
-      <c r="E24" s="1">
-        <v>9</v>
-      </c>
-      <c r="F24" s="1">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>1</v>
-      </c>
-      <c r="B25" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="C25" s="1">
-        <v>5</v>
-      </c>
-      <c r="D25" s="1">
-        <v>21</v>
-      </c>
-      <c r="E25" s="1">
-        <v>24</v>
-      </c>
-      <c r="F25" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>1</v>
-      </c>
-      <c r="B26" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C26" s="1">
-        <v>25</v>
-      </c>
-      <c r="D26" s="1">
-        <v>35</v>
-      </c>
-      <c r="E26" s="1">
-        <v>41</v>
-      </c>
-      <c r="F26" s="1">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>1</v>
-      </c>
-      <c r="B27" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C27" s="2">
-        <f>SUM(C13:C26)</f>
-        <v>116</v>
-      </c>
-      <c r="D27" s="2">
-        <f>SUM(D13:D26)</f>
-        <v>213</v>
-      </c>
-      <c r="E27" s="2">
-        <f>SUM(E13:E26)</f>
-        <v>273</v>
-      </c>
-      <c r="F27" s="2">
-        <f>SUM(F13:F26)</f>
-        <v>321</v>
-      </c>
-      <c r="G27" s="2">
-        <f t="shared" ref="G27:J27" si="2">SUM(G13:G26)</f>
-        <v>0</v>
-      </c>
-      <c r="H27" s="2">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I27" s="2">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J27" s="2">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>1</v>
-      </c>
-      <c r="B28" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="C28" s="2">
-        <f>SUM(C13:C26)-C26</f>
-        <v>91</v>
-      </c>
-      <c r="D28" s="2">
-        <f>SUM(D13:D26)-D26</f>
-        <v>178</v>
-      </c>
-      <c r="E28" s="2">
-        <f>SUM(E13:E26)-E26</f>
-        <v>232</v>
-      </c>
-      <c r="F28" s="2">
-        <f>SUM(F13:F26)-F26</f>
-        <v>246</v>
-      </c>
-      <c r="G28" s="2">
-        <f t="shared" ref="G28:J28" si="3">SUM(G13:G26)-G26</f>
-        <v>0</v>
-      </c>
-      <c r="H28" s="2">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="I28" s="2">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J28" s="2">
-        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -4676,4 +5059,244 @@
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3E93DFC-AF79-47E5-9301-280331A46C77}">
+  <dimension ref="A1:J12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="25.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="I1" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="J1" s="14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A2" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" s="27"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="27">
+        <v>2</v>
+      </c>
+      <c r="I2" s="28"/>
+      <c r="J2" s="29"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A3" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="1"/>
+      <c r="H3" s="1">
+        <v>1</v>
+      </c>
+      <c r="J3" s="30"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A4" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="18"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="18"/>
+      <c r="H4" s="19">
+        <f>SUM(H2:H3)</f>
+        <v>3</v>
+      </c>
+      <c r="I4" s="18"/>
+      <c r="J4" s="31"/>
+    </row>
+    <row r="5" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="23">
+        <f>SUM(H2:H3)-H3</f>
+        <v>2</v>
+      </c>
+      <c r="I5" s="22"/>
+      <c r="J5" s="32"/>
+    </row>
+    <row r="6" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="7" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="34" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="35" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="36" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="36" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" s="36" t="s">
+        <v>23</v>
+      </c>
+      <c r="G7" s="36" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" s="36" t="s">
+        <v>25</v>
+      </c>
+      <c r="I7" s="36" t="s">
+        <v>26</v>
+      </c>
+      <c r="J7" s="37" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27">
+        <v>1</v>
+      </c>
+      <c r="I8" s="27"/>
+      <c r="J8" s="33"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1">
+        <v>1</v>
+      </c>
+      <c r="I9" s="1"/>
+      <c r="J9" s="17"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1">
+        <v>1</v>
+      </c>
+      <c r="I10" s="1"/>
+      <c r="J10" s="17"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="19">
+        <f>SUM(H8:H10)</f>
+        <v>3</v>
+      </c>
+      <c r="I11" s="18"/>
+      <c r="J11" s="31"/>
+    </row>
+    <row r="12" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="22"/>
+      <c r="H12" s="23">
+        <f>SUM(H8:H10)-H10</f>
+        <v>2</v>
+      </c>
+      <c r="I12" s="22"/>
+      <c r="J12" s="32"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
chore: subir últimos cambios (index.html, wram/index.html, Excel actualizado)
</commit_message>
<xml_diff>
--- a/Presentación Semanal UAT.xlsx
+++ b/Presentación Semanal UAT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\QA\WrampUp - copia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A7EC188-9DBA-45C5-9F51-38445C80005F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7526D54-778D-449B-8E81-43BEDD005CA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{27A98AC9-9505-493B-985E-2D79FFCBCA40}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="52">
   <si>
     <t>Aplicación</t>
   </si>
@@ -591,13 +591,13 @@
                   <c:v>93</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>70</c:v>
+                  <c:v>57</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>47</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>24</c:v>
+                  <c:v>11</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -795,7 +795,10 @@
                   <c:v>116</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>86</c:v>
+                  <c:v>80</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>49</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3622,11 +3625,11 @@
         <v>328</v>
       </c>
       <c r="C2" s="5">
-        <v>202</v>
+        <v>186</v>
       </c>
       <c r="D2" s="6">
         <f>(C2*100)/B2</f>
-        <v>61.585365853658537</v>
+        <v>56.707317073170735</v>
       </c>
       <c r="E2" s="5">
         <v>1049</v>
@@ -3643,14 +3646,14 @@
         <v>46</v>
       </c>
       <c r="C3" s="5">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D3" s="6">
         <f>(C3*100)/B3</f>
-        <v>10.869565217391305</v>
+        <v>15.217391304347826</v>
       </c>
       <c r="E3" s="5">
-        <v>74</v>
+        <v>18</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>9</v>
@@ -3664,11 +3667,11 @@
         <v>82</v>
       </c>
       <c r="C4" s="5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D4" s="6">
         <f t="shared" ref="D4:D5" si="0">(C4*100)/B4</f>
-        <v>8.536585365853659</v>
+        <v>7.3170731707317076</v>
       </c>
       <c r="E4" s="5">
         <v>154</v>
@@ -3706,7 +3709,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42DF1849-A1A9-4E05-97A1-E2B79B421503}">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.36328125" bestFit="1" customWidth="1"/>
@@ -3858,13 +3861,13 @@
       </c>
       <c r="D7" s="5">
         <f>D6-F7</f>
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="E7" s="5">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F7" s="5">
-        <v>30</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
@@ -3875,14 +3878,19 @@
         <v>1</v>
       </c>
       <c r="C8" s="5">
-        <f t="shared" ref="C5:C11" si="0">C7-$E$2</f>
-        <v>70</v>
-      </c>
-      <c r="D8" s="5"/>
+        <f>C7-20-16</f>
+        <v>57</v>
+      </c>
+      <c r="D8" s="5">
+        <f>D7-F8-16</f>
+        <v>49</v>
+      </c>
       <c r="E8" s="5">
-        <v>23</v>
-      </c>
-      <c r="F8" s="5"/>
+        <v>20</v>
+      </c>
+      <c r="F8" s="5">
+        <v>15</v>
+      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
@@ -3892,12 +3900,12 @@
         <v>1</v>
       </c>
       <c r="C9" s="5">
-        <f t="shared" si="0"/>
-        <v>47</v>
+        <f t="shared" ref="C9:C11" si="0">C8-$E$2</f>
+        <v>34</v>
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="5">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F9" s="5"/>
     </row>
@@ -3910,11 +3918,11 @@
       </c>
       <c r="C10" s="5">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="5">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F10" s="5"/>
     </row>
@@ -3927,11 +3935,11 @@
       </c>
       <c r="C11" s="5">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>-12</v>
       </c>
       <c r="D11" s="5"/>
       <c r="E11" s="5">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F11" s="5"/>
     </row>
@@ -3991,6 +3999,118 @@
         <v>4</v>
       </c>
       <c r="F14" s="5"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" s="4">
+        <v>0</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="5">
+        <v>6</v>
+      </c>
+      <c r="D15" s="5">
+        <v>6</v>
+      </c>
+      <c r="E15" s="5">
+        <v>3</v>
+      </c>
+      <c r="F15" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" s="4">
+        <v>1</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" s="5">
+        <v>3</v>
+      </c>
+      <c r="D16" s="5">
+        <v>1</v>
+      </c>
+      <c r="E16" s="5">
+        <v>3</v>
+      </c>
+      <c r="F16" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" s="4">
+        <v>2</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" s="5">
+        <v>3</v>
+      </c>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5">
+        <v>3</v>
+      </c>
+      <c r="F17" s="5"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A18" s="4">
+        <v>0</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" s="5">
+        <v>7</v>
+      </c>
+      <c r="D18" s="5">
+        <v>7</v>
+      </c>
+      <c r="E18" s="5">
+        <v>3</v>
+      </c>
+      <c r="F18" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A19" s="4">
+        <v>1</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" s="5">
+        <v>4</v>
+      </c>
+      <c r="D19" s="5">
+        <v>0</v>
+      </c>
+      <c r="E19" s="5">
+        <v>3</v>
+      </c>
+      <c r="F19" s="5">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" s="4">
+        <v>2</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="5">
+        <v>3</v>
+      </c>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5">
+        <v>3</v>
+      </c>
+      <c r="F20" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4356,6 +4476,9 @@
       <c r="G2" s="1">
         <v>12</v>
       </c>
+      <c r="H2" s="1">
+        <v>15</v>
+      </c>
       <c r="J2" s="17"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
@@ -4380,6 +4503,9 @@
       <c r="G3" s="1">
         <v>81</v>
       </c>
+      <c r="H3" s="1">
+        <v>86</v>
+      </c>
       <c r="J3" s="17"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
@@ -4404,6 +4530,9 @@
       <c r="G4" s="1">
         <v>13</v>
       </c>
+      <c r="H4" s="1">
+        <v>54</v>
+      </c>
       <c r="J4" s="17"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
@@ -4428,6 +4557,9 @@
       <c r="G5" s="1">
         <v>45</v>
       </c>
+      <c r="H5" s="1">
+        <v>45</v>
+      </c>
       <c r="J5" s="17"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
@@ -4452,6 +4584,9 @@
       <c r="G6" s="1">
         <v>85</v>
       </c>
+      <c r="H6" s="1">
+        <v>90</v>
+      </c>
       <c r="J6" s="17"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
@@ -4476,6 +4611,9 @@
       <c r="G7" s="1">
         <v>0</v>
       </c>
+      <c r="H7" s="1">
+        <v>0</v>
+      </c>
       <c r="J7" s="17"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
@@ -4500,6 +4638,9 @@
       <c r="G8" s="1">
         <v>0</v>
       </c>
+      <c r="H8" s="1">
+        <v>0</v>
+      </c>
       <c r="J8" s="17"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
@@ -4524,6 +4665,9 @@
       <c r="G9" s="1">
         <v>101</v>
       </c>
+      <c r="H9" s="1">
+        <v>109</v>
+      </c>
       <c r="J9" s="17"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
@@ -4534,28 +4678,28 @@
         <v>19</v>
       </c>
       <c r="C10" s="19">
-        <f>SUM(C2:C9)</f>
+        <f t="shared" ref="C10:H10" si="0">SUM(C2:C9)</f>
         <v>116</v>
       </c>
       <c r="D10" s="19">
-        <f>SUM(D2:D9)</f>
+        <f t="shared" si="0"/>
         <v>213</v>
       </c>
       <c r="E10" s="19">
-        <f>SUM(E2:E9)</f>
+        <f t="shared" si="0"/>
         <v>273</v>
       </c>
       <c r="F10" s="19">
-        <f>SUM(F2:F9)</f>
+        <f t="shared" si="0"/>
         <v>321</v>
       </c>
       <c r="G10" s="19">
-        <f>SUM(G2:G9)</f>
+        <f t="shared" si="0"/>
         <v>337</v>
       </c>
       <c r="H10" s="19">
-        <f>SUM(H4:H9)</f>
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>399</v>
       </c>
       <c r="I10" s="19">
         <f>SUM(I4:I9)</f>
@@ -4574,28 +4718,28 @@
         <v>35</v>
       </c>
       <c r="C11" s="19">
-        <f>SUM(C2:C9)-C9</f>
+        <f t="shared" ref="C11:H11" si="1">SUM(C2:C9)-C9</f>
         <v>91</v>
       </c>
       <c r="D11" s="19">
-        <f>SUM(D2:D9)-D9</f>
+        <f t="shared" si="1"/>
         <v>178</v>
       </c>
       <c r="E11" s="19">
-        <f>SUM(E2:E9)-E9</f>
+        <f t="shared" si="1"/>
         <v>232</v>
       </c>
       <c r="F11" s="19">
-        <f>SUM(F2:F9)-F9</f>
+        <f t="shared" si="1"/>
         <v>246</v>
       </c>
       <c r="G11" s="19">
-        <f>SUM(G2:G9)-G9</f>
+        <f t="shared" si="1"/>
         <v>236</v>
       </c>
       <c r="H11" s="19">
-        <f>SUM(H4:H9)-H9</f>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>290</v>
       </c>
       <c r="I11" s="19">
         <f>SUM(I4:I9)-I9</f>
@@ -4661,6 +4805,9 @@
       <c r="G14" s="1">
         <v>49</v>
       </c>
+      <c r="H14" s="1">
+        <v>48</v>
+      </c>
       <c r="J14" s="17"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
@@ -4685,6 +4832,9 @@
       <c r="G15" s="1">
         <v>9</v>
       </c>
+      <c r="H15" s="1">
+        <v>9</v>
+      </c>
       <c r="J15" s="17"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
@@ -4709,6 +4859,9 @@
       <c r="G16" s="1">
         <v>23</v>
       </c>
+      <c r="H16" s="1">
+        <v>20</v>
+      </c>
       <c r="J16" s="17"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
@@ -4733,6 +4886,9 @@
       <c r="G17" s="1">
         <v>14</v>
       </c>
+      <c r="H17" s="1">
+        <v>13</v>
+      </c>
       <c r="J17" s="17"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
@@ -4757,6 +4913,9 @@
       <c r="G18" s="1">
         <v>8</v>
       </c>
+      <c r="H18" s="1">
+        <v>10</v>
+      </c>
       <c r="J18" s="17"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
@@ -4781,6 +4940,9 @@
       <c r="G19" s="1">
         <v>34</v>
       </c>
+      <c r="H19" s="1">
+        <v>34</v>
+      </c>
       <c r="J19" s="17"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
@@ -4805,6 +4967,9 @@
       <c r="G20" s="1">
         <v>2</v>
       </c>
+      <c r="H20" s="1">
+        <v>2</v>
+      </c>
       <c r="J20" s="17"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
@@ -4829,6 +4994,9 @@
       <c r="G21" s="1">
         <v>3</v>
       </c>
+      <c r="H21" s="1">
+        <v>3</v>
+      </c>
       <c r="J21" s="17"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.35">
@@ -4853,6 +5021,9 @@
       <c r="G22" s="1">
         <v>26</v>
       </c>
+      <c r="H22" s="1">
+        <v>26</v>
+      </c>
       <c r="J22" s="17"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
@@ -4877,6 +5048,9 @@
       <c r="G23" s="1">
         <v>21</v>
       </c>
+      <c r="H23" s="1">
+        <v>21</v>
+      </c>
       <c r="J23" s="17"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.35">
@@ -4901,6 +5075,9 @@
       <c r="G24" s="1">
         <v>38</v>
       </c>
+      <c r="H24" s="1">
+        <v>37</v>
+      </c>
       <c r="J24" s="17"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
@@ -4925,6 +5102,9 @@
       <c r="G25" s="1">
         <v>9</v>
       </c>
+      <c r="H25" s="1">
+        <v>8</v>
+      </c>
       <c r="J25" s="17"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.35">
@@ -4949,6 +5129,9 @@
       <c r="G26" s="1">
         <v>0</v>
       </c>
+      <c r="H26" s="1">
+        <v>0</v>
+      </c>
       <c r="J26" s="17"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.35">
@@ -4973,6 +5156,9 @@
       <c r="G27" s="1">
         <v>101</v>
       </c>
+      <c r="H27" s="1">
+        <v>109</v>
+      </c>
       <c r="J27" s="17"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.35">
@@ -4983,35 +5169,35 @@
         <v>19</v>
       </c>
       <c r="C28" s="19">
-        <f t="shared" ref="C28:J28" si="0">SUM(C14:C27)</f>
+        <f t="shared" ref="C28:J28" si="2">SUM(C14:C27)</f>
         <v>116</v>
       </c>
       <c r="D28" s="19">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>213</v>
       </c>
       <c r="E28" s="19">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>273</v>
       </c>
       <c r="F28" s="19">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>321</v>
       </c>
       <c r="G28" s="19">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>337</v>
       </c>
       <c r="H28" s="19">
-        <f t="shared" si="0"/>
+        <f>SUM(H14:H27)</f>
+        <v>340</v>
+      </c>
+      <c r="I28" s="19">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="I28" s="19">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
       <c r="J28" s="20">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -5023,35 +5209,35 @@
         <v>35</v>
       </c>
       <c r="C29" s="23">
-        <f t="shared" ref="C29:J29" si="1">SUM(C14:C27)-C27</f>
+        <f t="shared" ref="C29:J29" si="3">SUM(C14:C27)-C27</f>
         <v>91</v>
       </c>
       <c r="D29" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>178</v>
       </c>
       <c r="E29" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>232</v>
       </c>
       <c r="F29" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>246</v>
       </c>
       <c r="G29" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>236</v>
       </c>
       <c r="H29" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
+        <v>231</v>
+      </c>
+      <c r="I29" s="23">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="I29" s="23">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
       <c r="J29" s="24">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -5115,7 +5301,7 @@
       <c r="F2" s="28"/>
       <c r="G2" s="28"/>
       <c r="H2" s="27">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I2" s="28"/>
       <c r="J2" s="29"/>
@@ -5129,7 +5315,7 @@
       </c>
       <c r="C3" s="1"/>
       <c r="H3" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J3" s="30"/>
     </row>
@@ -5166,7 +5352,7 @@
       <c r="G5" s="22"/>
       <c r="H5" s="23">
         <f>SUM(H2:H3)-H3</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I5" s="22"/>
       <c r="J5" s="32"/>
@@ -5217,7 +5403,7 @@
       <c r="F8" s="27"/>
       <c r="G8" s="27"/>
       <c r="H8" s="27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I8" s="27"/>
       <c r="J8" s="33"/>
@@ -5235,7 +5421,7 @@
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I9" s="1"/>
       <c r="J9" s="17"/>
@@ -5253,7 +5439,7 @@
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
       <c r="H10" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="17"/>
@@ -5291,7 +5477,7 @@
       <c r="G12" s="22"/>
       <c r="H12" s="23">
         <f>SUM(H8:H10)-H10</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I12" s="22"/>
       <c r="J12" s="32"/>

</xml_diff>